<commit_message>
The update and hashing implemented
</commit_message>
<xml_diff>
--- a/data/sales-tracker.xlsx
+++ b/data/sales-tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/realdekings/Documents/Projects/data-engineering/small-business-sales-tracker-pipeline/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47518805-88DA-5D44-ADD5-5E4CC499B7B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD050880-FE4F-E34A-8739-8660082F1F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SalesTracker" sheetId="1" r:id="rId1"/>
@@ -1790,9 +1790,6 @@
     <t>$15.00</t>
   </si>
   <si>
-    <t>$105.00</t>
-  </si>
-  <si>
     <t>$25.00</t>
   </si>
   <si>
@@ -1833,6 +1830,9 @@
   </si>
   <si>
     <t>$168.00</t>
+  </si>
+  <si>
+    <t>$100.00</t>
   </si>
 </sst>
 </file>
@@ -17174,10 +17174,10 @@
         <v>584</v>
       </c>
       <c r="H502" s="4">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I502" s="6" t="s">
-        <v>585</v>
+        <v>599</v>
       </c>
     </row>
     <row r="503" spans="1:9" x14ac:dyDescent="0.2">
@@ -17200,13 +17200,13 @@
         <v>13</v>
       </c>
       <c r="G503" s="6" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="H503" s="4">
         <v>1</v>
       </c>
       <c r="I503" s="6" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="504" spans="1:9" x14ac:dyDescent="0.2">
@@ -17229,13 +17229,13 @@
         <v>21</v>
       </c>
       <c r="G504" s="6" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="H504" s="4">
         <v>9</v>
       </c>
       <c r="I504" s="6" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="505" spans="1:9" x14ac:dyDescent="0.2">
@@ -17258,13 +17258,13 @@
         <v>24</v>
       </c>
       <c r="G505" s="6" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="H505" s="4">
         <v>8</v>
       </c>
       <c r="I505" s="6" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="506" spans="1:9" x14ac:dyDescent="0.2">
@@ -17287,13 +17287,13 @@
         <v>24</v>
       </c>
       <c r="G506" s="6" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="H506" s="4">
         <v>8</v>
       </c>
       <c r="I506" s="6" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="507" spans="1:9" x14ac:dyDescent="0.2">
@@ -17316,13 +17316,13 @@
         <v>21</v>
       </c>
       <c r="G507" s="6" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="H507" s="4">
         <v>8</v>
       </c>
       <c r="I507" s="6" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="508" spans="1:9" x14ac:dyDescent="0.2">
@@ -17345,13 +17345,13 @@
         <v>65</v>
       </c>
       <c r="G508" s="6" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="H508" s="4">
         <v>6</v>
       </c>
       <c r="I508" s="6" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="509" spans="1:9" x14ac:dyDescent="0.2">
@@ -17374,13 +17374,13 @@
         <v>21</v>
       </c>
       <c r="G509" s="6" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="H509" s="4">
         <v>5</v>
       </c>
       <c r="I509" s="6" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="510" spans="1:9" x14ac:dyDescent="0.2">
@@ -17409,7 +17409,7 @@
         <v>9</v>
       </c>
       <c r="I510" s="6" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="511" spans="1:9" x14ac:dyDescent="0.2">
@@ -17432,13 +17432,13 @@
         <v>21</v>
       </c>
       <c r="G511" s="6" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="H511" s="4">
         <v>4</v>
       </c>
       <c r="I511" s="6" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
     </row>
   </sheetData>

</xml_diff>